<commit_message>
nouvelle version de l'ig généré
</commit_message>
<xml_diff>
--- a/docs/StructureDefinition-fr-core-address-insee-code.xlsx
+++ b/docs/StructureDefinition-fr-core-address-insee-code.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-06-03T19:04:37+02:00</t>
+    <t>2025-11-02T16:31:57+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -681,40 +681,40 @@
   <cols>
     <col min="1" max="1" width="17.4375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.4375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="10.53125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="7.12890625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="5" max="5" width="5.65234375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="4.25" customWidth="true" bestFit="true"/>
-    <col min="7" max="7" width="4.625" customWidth="true" bestFit="true"/>
-    <col min="8" max="8" width="13.57421875" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.14453125" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.55859375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="7.17578125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="5" max="5" width="5.62890625" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="4.2421875" customWidth="true" bestFit="true"/>
+    <col min="7" max="7" width="4.640625" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="13.58984375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="11.17578125" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="11" max="11" width="8.93359375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
-    <col min="15" max="15" width="13.18359375" customWidth="true" bestFit="true"/>
+    <col min="15" max="15" width="13.23828125" customWidth="true" bestFit="true"/>
     <col min="16" max="16" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="17" max="17" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="18" max="18" width="20.703125" customWidth="true" bestFit="true"/>
     <col min="19" max="19" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="20" max="20" width="8.375" customWidth="true" bestFit="true"/>
-    <col min="21" max="21" width="14.54296875" customWidth="true" bestFit="true"/>
-    <col min="22" max="22" width="14.91796875" customWidth="true" bestFit="true"/>
-    <col min="23" max="23" width="16.1953125" customWidth="true" bestFit="true"/>
-    <col min="24" max="24" width="15.7578125" customWidth="true" bestFit="true"/>
-    <col min="25" max="25" width="18.1640625" customWidth="true" bestFit="true"/>
+    <col min="20" max="20" width="8.34765625" customWidth="true" bestFit="true"/>
+    <col min="21" max="21" width="14.65234375" customWidth="true" bestFit="true"/>
+    <col min="22" max="22" width="15.05078125" customWidth="true" bestFit="true"/>
+    <col min="23" max="23" width="16.32421875" customWidth="true" bestFit="true"/>
+    <col min="24" max="24" width="15.765625" customWidth="true" bestFit="true"/>
+    <col min="25" max="25" width="18.10546875" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="46.828125" customWidth="true" bestFit="true"/>
-    <col min="27" max="27" width="5.41015625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="18.95703125" customWidth="true" bestFit="true"/>
+    <col min="27" max="27" width="5.30078125" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="18.9921875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.56640625" customWidth="true" bestFit="true"/>
-    <col min="30" max="30" width="14.42578125" customWidth="true" bestFit="true"/>
-    <col min="31" max="31" width="11.828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="30" max="30" width="14.30859375" customWidth="true" bestFit="true"/>
+    <col min="31" max="31" width="11.7890625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="32" max="32" width="16.16015625" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="33" max="33" width="8.86328125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="34" max="34" width="9.23828125" customWidth="true" bestFit="true"/>
+    <col min="33" max="33" width="8.828125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="34" max="34" width="9.2265625" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="21.2421875" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="21.15234375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>